<commit_message>
Update ADS4229 register naming
</commit_message>
<xml_diff>
--- a/ads4229_register_map.xlsx
+++ b/ads4229_register_map.xlsx
@@ -2448,7 +2448,7 @@
     <row r="98">
       <c r="A98" s="20" t="inlineStr">
         <is>
-          <t>PA_DELAY_effect_0</t>
+          <t>PA_DELAY_EFFECT_0</t>
         </is>
       </c>
       <c r="B98" s="21" t="str">
@@ -3030,7 +3030,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>PA_DELAY_effect_1</t>
+          <t>PA_DELAY_EFFECT_1</t>
         </is>
       </c>
       <c r="B130" s="3" t="str">
@@ -3612,7 +3612,7 @@
     <row r="162">
       <c r="A162" s="20" t="inlineStr">
         <is>
-          <t>PA_DELAY_effect_2</t>
+          <t>PA_DELAY_EFFECT_2</t>
         </is>
       </c>
       <c r="B162" s="21" t="str">
@@ -5940,7 +5940,7 @@
     <row r="290">
       <c r="A290" s="20" t="inlineStr">
         <is>
-          <t>PB_DELAY_effect_0</t>
+          <t>PB_DELAY_EFFECT_0</t>
         </is>
       </c>
       <c r="B290" s="21" t="str">
@@ -6522,7 +6522,7 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>PB_DELAY_effect_1</t>
+          <t>PB_DELAY_EFFECT_1</t>
         </is>
       </c>
       <c r="B322" s="3" t="str">
@@ -7104,7 +7104,7 @@
     <row r="354">
       <c r="A354" s="20" t="inlineStr">
         <is>
-          <t>PB_DELAY_effect_2</t>
+          <t>PB_DELAY_EFFECT_2</t>
         </is>
       </c>
       <c r="B354" s="21" t="str">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="G64" s="12" t="inlineStr">
         <is>
-          <t>adc_poweren</t>
+          <t>adc_power_en</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="G18" s="26" t="inlineStr">
         <is>
-          <t>accmulator_status</t>
+          <t>accumulator_status</t>
         </is>
       </c>
       <c r="H18" s="27" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="G33" s="32" t="inlineStr">
         <is>
-          <t>accmulator_start</t>
+          <t>accumulator_start</t>
         </is>
       </c>
       <c r="H33" s="33" t="inlineStr">
@@ -15636,7 +15636,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>DATA_PRE_SAMPLE</t>
+          <t>DATA_POINTS_PER_SAMPLE</t>
         </is>
       </c>
       <c r="B66" s="3" t="str">
@@ -15794,7 +15794,7 @@
       </c>
       <c r="G74" s="12" t="inlineStr">
         <is>
-          <t>data_pre_sample</t>
+          <t>data_points_per_sample</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
@@ -16163,7 +16163,7 @@
     <row r="98">
       <c r="A98" s="20" t="inlineStr">
         <is>
-          <t>DATA_PRE_SLICE</t>
+          <t>DATA_POINTS_PER_SLICE</t>
         </is>
       </c>
       <c r="B98" s="21" t="str">
@@ -16321,7 +16321,7 @@
       </c>
       <c r="G106" s="12" t="inlineStr">
         <is>
-          <t>data_pre_slice</t>
+          <t>data_points_per_slice</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr">
@@ -16332,7 +16332,7 @@
       <c r="I106" s="14" t="inlineStr">
         <is>
           <t>每个 slice 采样的数据，配置值为实际值减一
-slice_pre_sample * data_pre_slice 必须等于 data_pre_sample</t>
+slices_per_sample * data_points_per_slice 必须等于 data_points_per_sample</t>
         </is>
       </c>
     </row>
@@ -16690,7 +16690,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>SAMPLE_PRE_BATCH</t>
+          <t>SAMPLES_PER_BATCH</t>
         </is>
       </c>
       <c r="B130" s="3" t="str">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="G138" s="12" t="inlineStr">
         <is>
-          <t>sample_pre_batch</t>
+          <t>samples_per_batch</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr">
@@ -17633,7 +17633,7 @@
       </c>
       <c r="G186" s="12" t="inlineStr">
         <is>
-          <t>slice_pre_sample</t>
+          <t>slices_per_sample</t>
         </is>
       </c>
       <c r="H186" s="13" t="inlineStr">
@@ -17645,7 +17645,7 @@
         <is>
           <t>一个 sample 内的 slice 数
 配置值为实际值减一
-slice_pre_sample % 2 == 0</t>
+slices_per_sample % 2 == 0</t>
         </is>
       </c>
     </row>
@@ -18834,7 +18834,7 @@
       </c>
       <c r="G258" s="35" t="inlineStr">
         <is>
-          <t>data_delay_pre_slice</t>
+          <t>data_delay_per_slice</t>
         </is>
       </c>
       <c r="H258" s="36" t="inlineStr">
@@ -18981,7 +18981,7 @@
         <is>
           <t>触发信号开始到下一次开始采样的延迟。
 配置值为实际值
-例如当 data_delay 配置为 5，data_delay_pre_slice 为1。Sample 开始时触发信号到开始采样的延迟为 5 ，当第一个 slice 完成，第二个 slice 开始时的延迟为 6，第三个为 7。在新的 sample 开始时，将清零</t>
+例如当 data_delay 配置为 5，data_delay_per_slice 为1。Sample 开始时触发信号到开始采样的延迟为 5 ，当第一个 slice 完成，第二个 slice 开始时的延迟为 6，第三个为 7。在新的 sample 开始时，将清零</t>
         </is>
       </c>
     </row>
@@ -19913,12 +19913,12 @@
           <t>每个 batch 累加结果存储的基地址
 每个 batch 存储值的 offset 与 RTL 配置相关
 OFFSET = 2 ^
-  CEIL(LOG2(MAX_DATA_PRE_SAMPLE)) * 4
+  CEIL(LOG2(MAX_DATA_POINTS_PER_SAMPLE)) * 4
 adc0 batch 结果存储在 batch_result_base_address，batch_result_base_address + OFFSET
 adc0 batch 结果存储在
  batch_result_base_address + OFFSET
  batch_result_base_address + 2 * OFFSET
-因此，需要保证 batch_result_base_address 到 batch_result_base_address + 2 * MAX_BATCHES * OFFSET 的地址段为空</t>
+因此，需要保证 batch_result_base_address 到 batch_result_base_address + 2 * MAX_BATCH_COUNT * OFFSET 的地址段为空</t>
         </is>
       </c>
     </row>
@@ -21181,7 +21181,7 @@
       </c>
       <c r="G398" s="26" t="inlineStr">
         <is>
-          <t>transfer_done_irq_flage</t>
+          <t>transfer_done_irq_flag</t>
         </is>
       </c>
       <c r="H398" s="27" t="inlineStr">
@@ -21208,7 +21208,7 @@
       </c>
       <c r="G399" s="26" t="inlineStr">
         <is>
-          <t>sample_done_irq_flage</t>
+          <t>sample_done_irq_flag</t>
         </is>
       </c>
       <c r="H399" s="27" t="inlineStr">
@@ -21231,7 +21231,7 @@
       </c>
       <c r="G400" s="26" t="inlineStr">
         <is>
-          <t>batch_done_irq_flage</t>
+          <t>batch_done_irq_flag</t>
         </is>
       </c>
       <c r="H400" s="27" t="inlineStr">
@@ -21254,7 +21254,7 @@
       </c>
       <c r="G401" s="26" t="inlineStr">
         <is>
-          <t>slice_done_irq_flage</t>
+          <t>slice_done_irq_flag</t>
         </is>
       </c>
       <c r="H401" s="27" t="inlineStr">

</xml_diff>